<commit_message>
More excel commands and some sql queries on Feb 27, 2022
</commit_message>
<xml_diff>
--- a/Excel/Excel_Commands.xlsx
+++ b/Excel/Excel_Commands.xlsx
@@ -1,31 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23801"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\IDM\Documents\Books\Excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8013BB4-B506-4A67-8FEF-B988B2744C30}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="22368" windowHeight="9215" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Excel Commands" sheetId="1" r:id="rId1"/>
+    <sheet name="Chrome Commands" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="175">
   <si>
     <t>Shortcut Keys</t>
   </si>
@@ -42,6 +32,9 @@
     <t>Ctrl + PageUP/Ctrl + PageDown</t>
   </si>
   <si>
+    <t>To goto other sheets in the workbook</t>
+  </si>
+  <si>
     <t>Shift + UP/Down/Left/Right Arrow</t>
   </si>
   <si>
@@ -60,12 +53,12 @@
     <t>To select a complete Column</t>
   </si>
   <si>
+    <t>Ctrl + Shift + Space/ Ctrl + A</t>
+  </si>
+  <si>
     <t>To select a complete sheet</t>
   </si>
   <si>
-    <t>Ctrl + Shift + Space/ Ctrl + A</t>
-  </si>
-  <si>
     <t>Home</t>
   </si>
   <si>
@@ -84,15 +77,15 @@
     <t>PageUP/PageDown</t>
   </si>
   <si>
+    <t>To scroll sheet up and down respectively</t>
+  </si>
+  <si>
     <t>Alt + PageUP/ Alt + PageDown</t>
   </si>
   <si>
     <t>To scroll sheet Right and Left respetively</t>
   </si>
   <si>
-    <t>To scroll sheet up and down respectively</t>
-  </si>
-  <si>
     <t>F8</t>
   </si>
   <si>
@@ -111,9 +104,6 @@
     <t>Insert a new sheet in the workbook</t>
   </si>
   <si>
-    <t>To goto other sheets in the workbook</t>
-  </si>
-  <si>
     <t>Ctrl + N</t>
   </si>
   <si>
@@ -213,15 +203,15 @@
     <t>Ctrl + 9</t>
   </si>
   <si>
+    <t>Hide row</t>
+  </si>
+  <si>
     <t>Ctrl + Shift + 9</t>
   </si>
   <si>
     <t>Unhide row</t>
   </si>
   <si>
-    <t>Hide row</t>
-  </si>
-  <si>
     <t>Ctrl + 0</t>
   </si>
   <si>
@@ -288,12 +278,12 @@
     <t>Fill Down</t>
   </si>
   <si>
+    <t>Ctrl + R</t>
+  </si>
+  <si>
     <t>Fill Right</t>
   </si>
   <si>
-    <t>Ctrl + R</t>
-  </si>
-  <si>
     <t>Ctrl + F10</t>
   </si>
   <si>
@@ -342,12 +332,12 @@
     <t>Current Date</t>
   </si>
   <si>
+    <t>Ctrl + Shift + :</t>
+  </si>
+  <si>
     <t>Current Time</t>
   </si>
   <si>
-    <t>Ctrl + Shift + :</t>
-  </si>
-  <si>
     <t>Ctrl + T/L</t>
   </si>
   <si>
@@ -418,36 +408,317 @@
   </si>
   <si>
     <t xml:space="preserve">To remove format </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ctrl + t</t>
+  </si>
+  <si>
+    <t>Open a new tab, and jump to it</t>
+  </si>
+  <si>
+    <t>Ctrl + Tab or Ctrl + PgDn</t>
+  </si>
+  <si>
+    <t>Jump to the next open tab</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + Tab or Ctrl + PgUp</t>
+  </si>
+  <si>
+    <t>Jump to the previous open tab</t>
+  </si>
+  <si>
+    <t>Ctrl + 1 through Ctrl + 8</t>
+  </si>
+  <si>
+    <t>Jump to a specific tab</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Alt + Home</t>
+  </si>
+  <si>
+    <t>Open your home page in the current tab</t>
+  </si>
+  <si>
+    <t>Alt + Left arrow</t>
+  </si>
+  <si>
+    <t>Open the previous page from your browsing history in the current tab</t>
+  </si>
+  <si>
+    <t>Alt + Right arrow</t>
+  </si>
+  <si>
+    <t>Open the next page from your browsing history in the current tab</t>
+  </si>
+  <si>
+    <t>Ctrl + Right arrow or Ctrl + Left arrow</t>
+  </si>
+  <si>
+    <t>Move tabs right or left with keyboard focus</t>
+  </si>
+  <si>
+    <t>Alt + f or Alt + e</t>
+  </si>
+  <si>
+    <t>Open the Chrome menu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ctrl + Shift + b</t>
+  </si>
+  <si>
+    <t>Show or hide the Bookmarks bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ctrl + Shift + o</t>
+  </si>
+  <si>
+    <t>Open the Bookmarks Manager</t>
+  </si>
+  <si>
+    <t>Shift + Esc</t>
+  </si>
+  <si>
+    <t>Open the Chrome Task Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ctrl + g</t>
+  </si>
+  <si>
+    <t>Jump to the next match to your Find Bar search</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + Delete</t>
+  </si>
+  <si>
+    <t>Open the Clear Browsing Data options</t>
+  </si>
+  <si>
+    <t>Type a search engine name and press Tab</t>
+  </si>
+  <si>
+    <t>Search using a different search engine</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ctrl + l or Alt + d or F6</t>
+  </si>
+  <si>
+    <t>Jump to the address bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ctrl + e</t>
+  </si>
+  <si>
+    <t>Search from anywhere on the page</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Control + F5</t>
+  </si>
+  <si>
+    <t>Move cursor to the address bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Type a search term + Alt + Enter</t>
+  </si>
+  <si>
+    <t>Open a new tab and perform a Google search</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> F5 or Ctrl + r</t>
+  </si>
+  <si>
+    <t>Reload the current page</t>
+  </si>
+  <si>
+    <t>Shift + F5 or Ctrl + Shift + r</t>
+  </si>
+  <si>
+    <t>Reload the current page, ignoring cached content</t>
+  </si>
+  <si>
+    <t>Shift + Scroll your mousewheel</t>
+  </si>
+  <si>
+    <t>Scroll horizontally on the page</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C5700"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Helvetica"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -457,10 +728,191 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -468,28 +920,311 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="30"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="3" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Currency" xfId="5" builtinId="4"/>
+    <cellStyle name="Percent" xfId="6" builtinId="5"/>
+    <cellStyle name="Hyperlink" xfId="7" builtinId="8"/>
+    <cellStyle name="60% - Accent4" xfId="8" builtinId="44"/>
+    <cellStyle name="Followed Hyperlink" xfId="9" builtinId="9"/>
+    <cellStyle name="Check Cell" xfId="10" builtinId="23"/>
+    <cellStyle name="Heading 2" xfId="11" builtinId="17"/>
+    <cellStyle name="Note" xfId="12" builtinId="10"/>
+    <cellStyle name="40% - Accent3" xfId="13" builtinId="39"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11"/>
+    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
+    <cellStyle name="Title" xfId="16" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="17" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="18" builtinId="16"/>
+    <cellStyle name="Heading 3" xfId="19" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="20" builtinId="19"/>
+    <cellStyle name="Input" xfId="21" builtinId="20"/>
+    <cellStyle name="60% - Accent3" xfId="22" builtinId="40"/>
+    <cellStyle name="Good" xfId="23" builtinId="26"/>
+    <cellStyle name="Output" xfId="24" builtinId="21"/>
+    <cellStyle name="20% - Accent1" xfId="25" builtinId="30"/>
+    <cellStyle name="Calculation" xfId="26" builtinId="22"/>
+    <cellStyle name="Linked Cell" xfId="27" builtinId="24"/>
+    <cellStyle name="Total" xfId="28" builtinId="25"/>
+    <cellStyle name="Bad" xfId="29" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="30" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="31" builtinId="29"/>
+    <cellStyle name="20% - Accent5" xfId="32" builtinId="46"/>
+    <cellStyle name="60% - Accent1" xfId="33" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="34" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="35" builtinId="34"/>
+    <cellStyle name="20% - Accent6" xfId="36" builtinId="50"/>
+    <cellStyle name="60% - Accent2" xfId="37" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="38" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="39" builtinId="38"/>
+    <cellStyle name="Accent4" xfId="40" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="41" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="42" builtinId="43"/>
+    <cellStyle name="Accent5" xfId="43" builtinId="45"/>
+    <cellStyle name="40% - Accent5" xfId="44" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="45" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="46" builtinId="49"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -538,7 +1273,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -573,7 +1308,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -747,25 +1482,20 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="60" customWidth="1"/>
     <col min="2" max="2" width="77" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" s="1" customFormat="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -773,7 +1503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -781,111 +1511,111 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>19</v>
-      </c>
       <c r="B12" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -893,7 +1623,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -901,7 +1631,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -909,7 +1639,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -917,7 +1647,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -925,7 +1655,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -933,7 +1663,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>41</v>
       </c>
@@ -941,7 +1671,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>43</v>
       </c>
@@ -949,7 +1679,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2">
       <c r="A24" t="s">
         <v>45</v>
       </c>
@@ -957,7 +1687,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2">
       <c r="A25" t="s">
         <v>47</v>
       </c>
@@ -965,7 +1695,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2">
       <c r="A26" t="s">
         <v>49</v>
       </c>
@@ -973,7 +1703,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2">
       <c r="A27" t="s">
         <v>51</v>
       </c>
@@ -981,7 +1711,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2">
       <c r="A28" t="s">
         <v>53</v>
       </c>
@@ -989,7 +1719,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2">
       <c r="A29" t="s">
         <v>55</v>
       </c>
@@ -997,7 +1727,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2">
       <c r="A30" t="s">
         <v>57</v>
       </c>
@@ -1005,7 +1735,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2">
       <c r="A31" t="s">
         <v>59</v>
       </c>
@@ -1013,23 +1743,23 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2">
       <c r="A32" t="s">
         <v>61</v>
       </c>
       <c r="B32" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>62</v>
-      </c>
-      <c r="B33" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2">
       <c r="A34" t="s">
         <v>65</v>
       </c>
@@ -1037,12 +1767,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:2">
       <c r="B35" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -1050,7 +1780,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2">
       <c r="A37" t="s">
         <v>69</v>
       </c>
@@ -1058,7 +1788,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2">
       <c r="A38" t="s">
         <v>71</v>
       </c>
@@ -1066,7 +1796,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2">
       <c r="A39" t="s">
         <v>73</v>
       </c>
@@ -1074,7 +1804,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2">
       <c r="A40" t="s">
         <v>75</v>
       </c>
@@ -1082,7 +1812,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2">
       <c r="A41" t="s">
         <v>77</v>
       </c>
@@ -1090,7 +1820,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2">
       <c r="A42" t="s">
         <v>79</v>
       </c>
@@ -1098,7 +1828,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -1106,7 +1836,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2">
       <c r="A44" t="s">
         <v>83</v>
       </c>
@@ -1114,7 +1844,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2">
       <c r="A45" t="s">
         <v>85</v>
       </c>
@@ -1122,15 +1852,15 @@
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2">
       <c r="A46" t="s">
+        <v>87</v>
+      </c>
+      <c r="B46" t="s">
         <v>88</v>
       </c>
-      <c r="B46" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:2">
       <c r="A47" t="s">
         <v>89</v>
       </c>
@@ -1138,7 +1868,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2">
       <c r="A48" t="s">
         <v>91</v>
       </c>
@@ -1146,7 +1876,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2">
       <c r="A49" t="s">
         <v>93</v>
       </c>
@@ -1154,7 +1884,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2">
       <c r="A50" t="s">
         <v>95</v>
       </c>
@@ -1162,7 +1892,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2">
       <c r="A51" t="s">
         <v>97</v>
       </c>
@@ -1170,7 +1900,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2">
       <c r="A52" t="s">
         <v>99</v>
       </c>
@@ -1178,7 +1908,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2">
       <c r="A53" t="s">
         <v>101</v>
       </c>
@@ -1186,7 +1916,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2">
       <c r="A54" t="s">
         <v>103</v>
       </c>
@@ -1194,15 +1924,15 @@
         <v>104</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2">
       <c r="A55" t="s">
+        <v>105</v>
+      </c>
+      <c r="B55" t="s">
         <v>106</v>
       </c>
-      <c r="B55" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:2">
       <c r="A56" t="s">
         <v>107</v>
       </c>
@@ -1210,7 +1940,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2">
       <c r="A57" t="s">
         <v>109</v>
       </c>
@@ -1218,7 +1948,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2">
       <c r="A58" t="s">
         <v>111</v>
       </c>
@@ -1226,7 +1956,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2">
       <c r="A59" t="s">
         <v>113</v>
       </c>
@@ -1234,7 +1964,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2">
       <c r="A60" t="s">
         <v>115</v>
       </c>
@@ -1242,7 +1972,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2">
       <c r="A61" t="s">
         <v>117</v>
       </c>
@@ -1250,7 +1980,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2">
       <c r="A62" t="s">
         <v>119</v>
       </c>
@@ -1258,7 +1988,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2">
       <c r="A63" t="s">
         <v>121</v>
       </c>
@@ -1266,7 +1996,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2">
       <c r="A64" t="s">
         <v>123</v>
       </c>
@@ -1274,15 +2004,15 @@
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" s="2" t="s">
+    <row r="65" spans="1:2">
+      <c r="A65" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B65" s="2" t="s">
+      <c r="B65" s="3" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2">
       <c r="A66" t="s">
         <v>127</v>
       </c>
@@ -1290,7 +2020,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2">
       <c r="A67" t="s">
         <v>129</v>
       </c>
@@ -1300,5 +2030,206 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="36.3333333333333" customWidth="1"/>
+    <col min="2" max="2" width="139.666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B12" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B13" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>161</v>
+      </c>
+      <c r="B17" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>163</v>
+      </c>
+      <c r="B18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>165</v>
+      </c>
+      <c r="B19" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>167</v>
+      </c>
+      <c r="B20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>169</v>
+      </c>
+      <c r="B21" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>171</v>
+      </c>
+      <c r="B22" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>173</v>
+      </c>
+      <c r="B23" t="s">
+        <v>174</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated excel on May 08, 2022
</commit_message>
<xml_diff>
--- a/Excel/Excel_Commands.xlsx
+++ b/Excel/Excel_Commands.xlsx
@@ -1,21 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20375"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Books\Excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3E822D-56FA-4968-BB84-AD98AE392C14}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="22368" windowHeight="9215" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22368" windowHeight="9240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Excel Commands" sheetId="1" r:id="rId1"/>
     <sheet name="Chrome Commands" sheetId="2" r:id="rId2"/>
+    <sheet name="IntelliJ Shortcuts" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="295">
   <si>
     <t>Shortcut Keys</t>
   </si>
@@ -540,24 +547,385 @@
   </si>
   <si>
     <t>Scroll horizontally on the page</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Shortcut</t>
+  </si>
+  <si>
+    <t>Activate/Toggle Project Panel</t>
+  </si>
+  <si>
+    <t>Alt 1</t>
+  </si>
+  <si>
+    <t>Take cursor back to Editor</t>
+  </si>
+  <si>
+    <t>Minimize current panel and take cursor back to Editor</t>
+  </si>
+  <si>
+    <t>Shift Esc</t>
+  </si>
+  <si>
+    <t>Alt F12</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Open Terminal</t>
+  </si>
+  <si>
+    <t>Open Next Project Window</t>
+  </si>
+  <si>
+    <t>Open Previous Project Window</t>
+  </si>
+  <si>
+    <t>Alt Ctrl ]</t>
+  </si>
+  <si>
+    <t>Alt Ctrl [</t>
+  </si>
+  <si>
+    <t>Expand Bottom Panel Size</t>
+  </si>
+  <si>
+    <t>Ctrl Shift Up</t>
+  </si>
+  <si>
+    <t>Shrink Bottom Panel Size</t>
+  </si>
+  <si>
+    <t>Ctrl Shift Down</t>
+  </si>
+  <si>
+    <t>Expand Left Panel Size</t>
+  </si>
+  <si>
+    <t>Shrink Left Panel Size</t>
+  </si>
+  <si>
+    <t>Ctrl Shift Right</t>
+  </si>
+  <si>
+    <t>Ctrl Shift Left</t>
+  </si>
+  <si>
+    <t>Open a class</t>
+  </si>
+  <si>
+    <t>Ctrl N</t>
+  </si>
+  <si>
+    <t>Open a file</t>
+  </si>
+  <si>
+    <t>Ctrl Shift N</t>
+  </si>
+  <si>
+    <t>Open anything (class, file, symbol)</t>
+  </si>
+  <si>
+    <t>Double Shift</t>
+  </si>
+  <si>
+    <t>Open Recent Files (allows for partial name, camel case, abbreviations and wildcards).</t>
+  </si>
+  <si>
+    <t>Ctrl E</t>
+  </si>
+  <si>
+    <t>Open Recently Edited Files</t>
+  </si>
+  <si>
+    <t>Ctrl Shift E</t>
+  </si>
+  <si>
+    <t>Create new file/package.</t>
+  </si>
+  <si>
+    <t>Alt Ins (within project panel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Imports - Or any errors where Intellij provides you with possible solutions</t>
+  </si>
+  <si>
+    <t>move between errors</t>
+  </si>
+  <si>
+    <t>f2</t>
+  </si>
+  <si>
+    <t>Rename variable/method/class</t>
+  </si>
+  <si>
+    <t>Shift + F6</t>
+  </si>
+  <si>
+    <t>Comment / Uncomment</t>
+  </si>
+  <si>
+    <t>Ctrl + /</t>
+  </si>
+  <si>
+    <t>Extract Variable</t>
+  </si>
+  <si>
+    <t>Alt + Ctrl + V</t>
+  </si>
+  <si>
+    <t>Extract Field</t>
+  </si>
+  <si>
+    <t>Ctrl + Alt + F</t>
+  </si>
+  <si>
+    <t>Extract Method</t>
+  </si>
+  <si>
+    <t>Ctrl + Alt + M</t>
+  </si>
+  <si>
+    <t>To replace existing word instead of appending</t>
+  </si>
+  <si>
+    <t>Tab</t>
+  </si>
+  <si>
+    <t>Split into variable and declaration</t>
+  </si>
+  <si>
+    <t>Join lines</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + J</t>
+  </si>
+  <si>
+    <t>Format code</t>
+  </si>
+  <si>
+    <t>Ctrl + Alt + L</t>
+  </si>
+  <si>
+    <t>Template for iterating</t>
+  </si>
+  <si>
+    <t>iter</t>
+  </si>
+  <si>
+    <t>Template for for-loop</t>
+  </si>
+  <si>
+    <t>Fori</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Template for main method </t>
+  </si>
+  <si>
+    <t>Psvm</t>
+  </si>
+  <si>
+    <t>Templates for if null and if not null</t>
+  </si>
+  <si>
+    <t>ifn, inn</t>
+  </si>
+  <si>
+    <t>Templates for System.out and System.err print</t>
+  </si>
+  <si>
+    <t>sout, serr</t>
+  </si>
+  <si>
+    <t>Show Parameters</t>
+  </si>
+  <si>
+    <t>Ctrl + P</t>
+  </si>
+  <si>
+    <t>Navigate to declaration (variable) or open class</t>
+  </si>
+  <si>
+    <t>Ctrl + B</t>
+  </si>
+  <si>
+    <t>Override parent methods</t>
+  </si>
+  <si>
+    <t>Ctrl + O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Display all methods of class </t>
+  </si>
+  <si>
+    <t>to show super class methods also</t>
+  </si>
+  <si>
+    <t>Ctrl + F12 again</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Move between methods </t>
+  </si>
+  <si>
+    <t>Alt + Up/Down arrow</t>
+  </si>
+  <si>
+    <t>Move one Word at a time</t>
+  </si>
+  <si>
+    <t>Ctrl + Left/Right</t>
+  </si>
+  <si>
+    <t>Delete one Word at a time</t>
+  </si>
+  <si>
+    <t>Ctrl + Backspace</t>
+  </si>
+  <si>
+    <t>Move line</t>
+  </si>
+  <si>
+    <t>Alt + Shift + Up/Down</t>
+  </si>
+  <si>
+    <t>Delete Line</t>
+  </si>
+  <si>
+    <t>Ctrl + Y</t>
+  </si>
+  <si>
+    <t>Duplicate Line</t>
+  </si>
+  <si>
+    <t>Select Next occurrence</t>
+  </si>
+  <si>
+    <t>Alt + J</t>
+  </si>
+  <si>
+    <t>Select All occurrences</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + Alt + J</t>
+  </si>
+  <si>
+    <t>Expand Selection</t>
+  </si>
+  <si>
+    <t>Ctrl + W</t>
+  </si>
+  <si>
+    <t>Shrink Selection</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + W</t>
+  </si>
+  <si>
+    <t>Toggle Case</t>
+  </si>
+  <si>
+    <t>Find in Project (then Tab, then Enter to open)</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + F</t>
+  </si>
+  <si>
+    <t>Replace (Alt + P, to replace one, Alt + A to replace all)</t>
+  </si>
+  <si>
+    <t>Run Menu</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + F10</t>
+  </si>
+  <si>
+    <t>Debugging</t>
+  </si>
+  <si>
+    <t>Run last app</t>
+  </si>
+  <si>
+    <t>Shift + F10</t>
+  </si>
+  <si>
+    <t>Debug Menu</t>
+  </si>
+  <si>
+    <t>Ctrl + Shift + F9</t>
+  </si>
+  <si>
+    <t>Debug last app</t>
+  </si>
+  <si>
+    <t>Shift + F9</t>
+  </si>
+  <si>
+    <t>Toggle Breakpoint</t>
+  </si>
+  <si>
+    <t>Ctrl + F8</t>
+  </si>
+  <si>
+    <t>Continue execution (until next debug)</t>
+  </si>
+  <si>
+    <t>F9</t>
+  </si>
+  <si>
+    <t>Next statement</t>
+  </si>
+  <si>
+    <t>Go inside method</t>
+  </si>
+  <si>
+    <t>Restart</t>
+  </si>
+  <si>
+    <t>Ctrl+F5</t>
+  </si>
+  <si>
+    <t>Force Stop</t>
+  </si>
+  <si>
+    <t>Ctrl+F2</t>
+  </si>
+  <si>
+    <t>Reload</t>
+  </si>
+  <si>
+    <t>Ctrl+F9</t>
+  </si>
+  <si>
+    <t>Evaluate expression</t>
+  </si>
+  <si>
+    <t>Alt+F8</t>
+  </si>
+  <si>
+    <t>Text Editing</t>
+  </si>
+  <si>
+    <t>Working with IntelliJ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="22">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -575,155 +943,23 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -733,186 +969,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -920,311 +982,36 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="30"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="3">
+    <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
-    <cellStyle name="Comma" xfId="2" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="3" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
-    <cellStyle name="Currency" xfId="5" builtinId="4"/>
-    <cellStyle name="Percent" xfId="6" builtinId="5"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8"/>
-    <cellStyle name="60% - Accent4" xfId="8" builtinId="44"/>
-    <cellStyle name="Followed Hyperlink" xfId="9" builtinId="9"/>
-    <cellStyle name="Check Cell" xfId="10" builtinId="23"/>
-    <cellStyle name="Heading 2" xfId="11" builtinId="17"/>
-    <cellStyle name="Note" xfId="12" builtinId="10"/>
-    <cellStyle name="40% - Accent3" xfId="13" builtinId="39"/>
-    <cellStyle name="Warning Text" xfId="14" builtinId="11"/>
-    <cellStyle name="40% - Accent2" xfId="15" builtinId="35"/>
-    <cellStyle name="Title" xfId="16" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="17" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="18" builtinId="16"/>
-    <cellStyle name="Heading 3" xfId="19" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="20" builtinId="19"/>
-    <cellStyle name="Input" xfId="21" builtinId="20"/>
-    <cellStyle name="60% - Accent3" xfId="22" builtinId="40"/>
-    <cellStyle name="Good" xfId="23" builtinId="26"/>
-    <cellStyle name="Output" xfId="24" builtinId="21"/>
-    <cellStyle name="20% - Accent1" xfId="25" builtinId="30"/>
-    <cellStyle name="Calculation" xfId="26" builtinId="22"/>
-    <cellStyle name="Linked Cell" xfId="27" builtinId="24"/>
-    <cellStyle name="Total" xfId="28" builtinId="25"/>
-    <cellStyle name="Bad" xfId="29" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="30" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="31" builtinId="29"/>
-    <cellStyle name="20% - Accent5" xfId="32" builtinId="46"/>
-    <cellStyle name="60% - Accent1" xfId="33" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="34" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="35" builtinId="34"/>
-    <cellStyle name="20% - Accent6" xfId="36" builtinId="50"/>
-    <cellStyle name="60% - Accent2" xfId="37" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="38" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="39" builtinId="38"/>
-    <cellStyle name="Accent4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="42" builtinId="43"/>
-    <cellStyle name="Accent5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - Accent5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="45" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1482,24 +1269,24 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B67"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="60" customWidth="1"/>
     <col min="2" max="2" width="77" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" s="2" customFormat="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1767,7 +1554,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="1:2">
       <c r="B35" t="s">
         <v>67</v>
       </c>
@@ -2004,11 +1791,11 @@
         <v>124</v>
       </c>
     </row>
-    <row r="65" spans="1:2">
-      <c r="A65" s="3" t="s">
+    <row r="65" spans="1:2" s="6" customFormat="1">
+      <c r="A65" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B65" s="3" t="s">
+      <c r="B65" s="6" t="s">
         <v>126</v>
       </c>
     </row>
@@ -2030,25 +1817,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="36.3333333333333" customWidth="1"/>
-    <col min="2" max="2" width="139.666666666667" customWidth="1"/>
+    <col min="1" max="1" width="36.33203125" customWidth="1"/>
+    <col min="2" max="2" width="139.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:2" s="2" customFormat="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2157,7 +1942,7 @@
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>157</v>
       </c>
       <c r="B15" t="s">
@@ -2230,6 +2015,541 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B66"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="113.5546875" customWidth="1"/>
+    <col min="2" max="2" width="41.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" s="1" customFormat="1">
+      <c r="A2" s="5" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B5" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" s="6" customFormat="1">
+      <c r="A6" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>188</v>
+      </c>
+      <c r="B9" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>190</v>
+      </c>
+      <c r="B10" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>193</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" s="6" customFormat="1">
+      <c r="A15" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" s="6" customFormat="1">
+      <c r="A16" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="6" customFormat="1">
+      <c r="A19" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="6" customFormat="1">
+      <c r="A20" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" s="6" customFormat="1">
+      <c r="A21" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" s="6" customFormat="1">
+      <c r="A23" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" s="6" customFormat="1">
+      <c r="A29" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" s="6" customFormat="1">
+      <c r="A35" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" s="6" customFormat="1">
+      <c r="A38" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" s="6" customFormat="1">
+      <c r="A40" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" s="1" customFormat="1">
+      <c r="A41" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="B41" s="5"/>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" s="6" customFormat="1">
+      <c r="A44" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" s="6" customFormat="1">
+      <c r="A46" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" s="6" customFormat="1">
+      <c r="A48" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" s="6" customFormat="1">
+      <c r="A49" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" s="6" customFormat="1">
+      <c r="A50" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" s="1" customFormat="1">
+      <c r="A54" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="B54" s="5"/>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" s="6" customFormat="1">
+      <c r="A59" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" s="6" customFormat="1">
+      <c r="A61" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" s="6" customFormat="1">
+      <c r="A66" s="6" t="s">
+        <v>291</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>292</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>